<commit_message>
Add initial lead data for 家纺 (16 leads) and 家具 (53 leads)
First monitoring runs for home textile and furniture industries:
- 家纺: 21 signals from Reddit, 9 new qualified leads
- 家具: 66 signals from Reddit, 53 qualified leads
- Excel daily reports generated for both industries
</commit_message>
<xml_diff>
--- a/monitor/output/采购意向日报_家纺_20260322.xlsx
+++ b/monitor/output/采购意向日报_家纺_20260322.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -435,7 +435,7 @@
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
@@ -704,7 +704,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>lead-home_textile-20260322-001</t>
+          <t>lead-home_textile-20260322-002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -714,32 +714,32 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-03-22T14:46:41.913216+00:00</t>
+          <t>2026-03-22T15:05:55.650355+00:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Canadian Injection Molding</t>
+          <t>Curtain suggestions</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>UnculturedSwineFlu</t>
+          <t>Key-Trainer9929</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>需小批量（500–1000件）定制注塑产品，寻找加拿大本地小型注塑企业合作</t>
+          <t>厨房窗用窗帘；需防潮（距水槽&lt;6英寸）；适配狭小、视觉杂乱空间；抗强光、隔热</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>加拿大个人用户计划小批量复刻某产品，正在寻找本地注塑厂承接试产订单。</t>
+          <t>美国用户急需解决厨房强日照问题，明确需定制化窗帘产品，强调安装环境特殊性（近水源、空间局促），采购意向较强。</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -760,14 +760,14 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/InjectionMolding/comments/1rvqlga/canadian_injection_molding/</t>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1s07qgi/curtain_suggestions/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>lead-home_textile-20260322-003</t>
+          <t>lead-home_textile-20260322-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -777,32 +777,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-03-22T14:47:33.810364+00:00</t>
+          <t>2026-03-22T15:06:20.870931+00:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>What software do you use for batch tracking/moulding sheets?</t>
+          <t>How do I find curtains/drapes for my 12' sliding glass doors??</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>AndyTheRanga</t>
+          <t>maxthechuck</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>澳洲本地注塑车间初创阶段；需批次追踪/模具管理软件；预算&lt;2000美元/年</t>
+          <t>12英尺滑动玻璃门用窗帘，需两片100英寸以上面板，强调尺寸适配与操作便捷性</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -812,25 +812,25 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>初创注塑厂寻求低成本生产管理软件，有明确B2B采购场景和预算范围，但非硬件采购。</t>
+          <t>用户明确寻找超宽幅窗帘，已尝试多渠道未果，处于积极采购决策阶段。</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>持续跟踪</t>
+          <t>立即联系</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/InjectionMolding/comments/1rca56a/what_software_do_you_use_for_batch/</t>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1rzzjv6/how_do_i_find_curtainsdrapes_for_my_12_sliding/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>lead-home_textile-20260322-006</t>
+          <t>lead-home_textile-20260322-007</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -840,32 +840,32 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-03-22T14:47:33.810364+00:00</t>
+          <t>2026-03-22T15:06:20.870931+00:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>What's the most user-friendly desktop injection molding unti?</t>
+          <t>How do you decide when something in your home actually needs changing?</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>ArvinAbadilla</t>
+          <t>Full-potential678</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>家庭作坊级DIY注塑；Rubik's cube枪套；Formlabs Rigid 10K打印模具；APSX-PIM V3 / Micromolder桌面机对比</t>
+          <t>现有窗帘不平整、褪色，计划更换；提及Alibaba及长度/颜色/面料/款式等选型维度</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>家庭创业项目评估桌面注塑方案，有真实采购倾向和初步选型，但规模小、决策链短。</t>
+          <t>用户已意识到窗帘需更换，正陷入选品决策，明确表达线上比价行为，采购意向强烈。</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -886,14 +886,14 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/InjectionMolding/comments/1r7evj2/whats_the_most_userfriendly_desktop_injection/</t>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1rzjsez/how_do_you_decide_when_something_in_your_home/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lead-home_textile-20260322-007</t>
+          <t>lead-home_textile-20260322-001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-03-22T14:48:00.183080+00:00</t>
+          <t>2026-03-22T14:46:41.913216+00:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Starting a small run custom packaging operation out of my garage, odes this setup make sense?</t>
+          <t>Canadian Injection Molding</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -918,17 +918,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>palladinla</t>
+          <t>UnculturedSwineFlu</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Haitian MA600 injection molding machine, HDPE trays, custom packaging inserts (foam, plastic trays, branded dividers), sourcing molds from Alibaba/Made-in-China, considering corrugated expansion</t>
+          <t>需小批量（500–1000件）定制注塑产品，寻找加拿大本地小型注塑企业合作</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>墨西哥车库式包装厂采购注塑机并寻求海外模具，关注成本与质量平衡，潜在延伸至软质家居包装（如靠垫内衬、布套包装），有一定家纺关联性。</t>
+          <t>加拿大个人用户计划小批量复刻某产品，正在寻找本地注塑厂承接试产订单。</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -949,7 +949,574 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
+          <t>https://www.reddit.com/r/InjectionMolding/comments/1rvqlga/canadian_injection_molding/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-003</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-03-22T14:47:33.810364+00:00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>What software do you use for batch tracking/moulding sheets?</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>AndyTheRanga</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>澳洲本地注塑车间初创阶段；需批次追踪/模具管理软件；预算&lt;2000美元/年</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>short_term</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>初创注塑厂寻求低成本生产管理软件，有明确B2B采购场景和预算范围，但非硬件采购。</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InjectionMolding/comments/1rca56a/what_software_do_you_use_for_batch/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-006</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-03-22T14:47:33.810364+00:00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>What's the most user-friendly desktop injection molding unti?</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ArvinAbadilla</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>家庭作坊级DIY注塑；Rubik's cube枪套；Formlabs Rigid 10K打印模具；APSX-PIM V3 / Micromolder桌面机对比</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>short_term</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>家庭创业项目评估桌面注塑方案，有真实采购倾向和初步选型，但规模小、决策链短。</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>立即联系</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/InjectionMolding/comments/1r7evj2/whats_the_most_userfriendly_desktop_injection/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-007</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-03-22T14:48:00.183080+00:00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Starting a small run custom packaging operation out of my garage, odes this setup make sense?</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>palladinla</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Haitian MA600 injection molding machine, HDPE trays, custom packaging inserts (foam, plastic trays, branded dividers), sourcing molds from Alibaba/Made-in-China, considering corrugated expansion</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>short_term</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>墨西哥车库式包装厂采购注塑机并寻求海外模具，关注成本与质量平衡，潜在延伸至软质家居包装（如靠垫内衬、布套包装），有一定家纺关联性。</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/r/manufacturing/comments/1rri7dd/starting_a_small_run_custom_packaging_operation/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-001</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-03-22T15:05:55.650355+00:00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Need advice for durable rugs</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Embarrassed_Jello123</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>耐用、防污、柔软、适合硬木地板的地毯；需耐 toddlers 和 dogs 使用；易清洁</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>short_term</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>一位美国家庭用户正在为有幼儿和宠物的客厅寻找高品质、耐用且柔软的地毯，已对现有网购产品失望，有明确采购需求但未指定数量或规格。</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1s0je8s/need_advice_for_durable_rugs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-003</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-03-22T15:05:55.650355+00:00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Decision paralysis</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PressureMurky2495</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>客厅地毯；偏好复古风格；尺寸需适配空间；倾向中性浅色系（米白/中性色）；需覆盖深色木质地板与家具</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>long_term</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>用户已更换多款地毯，正积极搜寻合适复古地毯，有明确品类、色彩、尺寸及风格需求，但采购节奏偏慢。</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1s0763g/decision_paralysis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-03-22T15:05:55.650355+00:00</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Curtain question</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>horsegirl_99</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>窗帘类型识别；需兼容带孔窗帘的挂钩配件（用于窗帘杆）</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>short_term</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>用户计划更换窗帘，但缺乏专业知识，主动询问窗帘类型及安装配件，处于采购前期准备阶段，有明确更换意图。</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1s05d6z/curtain_question/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-006</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-03-22T15:06:20.870931+00:00</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Need help with my bedroom</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>MarkOutrageous1191</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>卧室床品配色咨询，未指定材质、尺寸或数量</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>long_term</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>用户重建卧室环境，提及需搭配床品，但尚处风格探索阶段，无具体采购参数。</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1rzl617/need_help_with_my_bedroom/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-008</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-03-22T15:06:20.870931+00:00</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Help me choose throw pillows</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>chewyspreeee</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>为蓝色沙发挑选抱枕，关注色彩搭配</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>long_term</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>用户寻求软装搭配建议，抱枕属低单价高频次消费品类，有潜在采购可能但未进入执行阶段。</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1rzg2y4/help_me_choose_throw_pillows/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>lead-home_textile-20260322-009</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>reddit</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-03-22T15:06:20.870931+00:00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Hanging curtains</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>poopybutt_andvag</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>公寓窗帘安装受阻，尚未选定窗帘产品，仅讨论安装方式</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>short_term</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>用户处于窗帘采购前期（安装准备），虽未选款但已启动行动，具备转化潜力。</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>持续跟踪</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/HomeDecorating/comments/1rz7e86/hanging_curtains/</t>
         </is>
       </c>
     </row>

</xml_diff>